<commit_message>
Week 02 Day 01: Excel data cleaning and text functions
</commit_message>
<xml_diff>
--- a/Month-01-Excel/Week-01/Week-01-Project/Week-01-Project-01-Sales-Analysis.xlsx.xlsx
+++ b/Month-01-Excel/Week-01/Week-01-Project/Week-01-Project-01-Sales-Analysis.xlsx.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\4_MONTH\4-Month-Data-Analyst-Journey\Month-01-Excel\Week-01\Day-06-Project\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\4_MONTH\4-Month-Data-Analyst-Journey\Month-01-Excel\Week-01\Week-01-Project\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F4FBDE8E-EB1C-4686-81F5-05621CB8C29F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2B249D28-23E3-458C-921F-1E0A6997E9F0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -132,7 +132,7 @@
 </file>
 
 <file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
   <metadataTypes count="1">
     <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
   </metadataTypes>
@@ -496,14 +496,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="10" x14ac:knownFonts="1">
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -669,47 +662,44 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="1" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="1" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="1" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -992,7 +982,6 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <sheetPr filterMode="1"/>
   <dimension ref="A1:Q22"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -1009,19 +998,19 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:17" ht="21" x14ac:dyDescent="0.35">
-      <c r="A1" s="13" t="s">
+      <c r="A1" s="12" t="s">
         <v>33</v>
       </c>
-      <c r="B1" s="13"/>
-      <c r="C1" s="13"/>
-      <c r="D1" s="13"/>
-      <c r="E1" s="13"/>
-      <c r="F1" s="13"/>
-      <c r="H1" s="20" t="s">
+      <c r="B1" s="12"/>
+      <c r="C1" s="12"/>
+      <c r="D1" s="12"/>
+      <c r="E1" s="12"/>
+      <c r="F1" s="12"/>
+      <c r="H1" s="17" t="s">
         <v>60</v>
       </c>
-      <c r="I1" s="21"/>
-      <c r="J1" s="21"/>
+      <c r="I1" s="18"/>
+      <c r="J1" s="18"/>
     </row>
     <row r="2" spans="1:17" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
@@ -1042,23 +1031,23 @@
       <c r="F2" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="H2" s="18" t="s">
+      <c r="H2" s="5" t="s">
         <v>61</v>
       </c>
-      <c r="I2" s="19" t="s">
+      <c r="I2" s="5" t="s">
         <v>62</v>
       </c>
-      <c r="J2" s="19" t="s">
+      <c r="J2" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="M2" s="9" t="s">
+      <c r="M2" s="13" t="s">
         <v>34</v>
       </c>
-      <c r="N2" s="9"/>
-      <c r="P2" s="9" t="s">
+      <c r="N2" s="13"/>
+      <c r="P2" s="13" t="s">
         <v>48</v>
       </c>
-      <c r="Q2" s="9"/>
+      <c r="Q2" s="13"/>
     </row>
     <row r="3" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
@@ -1091,7 +1080,7 @@
         <f>IF(AND(D3&gt;=40000,E3&gt;=8000),"Strong Order","Normal Order")</f>
         <v>Strong Order</v>
       </c>
-      <c r="M3" s="11" t="s">
+      <c r="M3" s="8" t="s">
         <v>35</v>
       </c>
       <c r="N3" s="3">
@@ -1106,7 +1095,7 @@
         <v>391000</v>
       </c>
     </row>
-    <row r="4" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>9</v>
       </c>
@@ -1135,7 +1124,7 @@
         <f t="shared" ref="J4:J22" si="0">IF(AND(D4&gt;=40000,E4&gt;=8000),"Strong Order","Normal Order")</f>
         <v>Normal Order</v>
       </c>
-      <c r="M4" s="12" t="s">
+      <c r="M4" s="9" t="s">
         <v>36</v>
       </c>
       <c r="N4" s="3">
@@ -1145,12 +1134,12 @@
       <c r="P4" s="4" t="s">
         <v>50</v>
       </c>
-      <c r="Q4" s="14">
+      <c r="Q4" s="10">
         <f>AVERAGEIF(Category,"Furniture",Profit)</f>
         <v>5857.1428571428569</v>
       </c>
     </row>
-    <row r="5" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>12</v>
       </c>
@@ -1179,7 +1168,7 @@
         <f t="shared" si="0"/>
         <v>Normal Order</v>
       </c>
-      <c r="M5" s="12" t="s">
+      <c r="M5" s="9" t="s">
         <v>37</v>
       </c>
       <c r="N5" s="3">
@@ -1216,7 +1205,7 @@
         <f t="shared" si="0"/>
         <v>Strong Order</v>
       </c>
-      <c r="M6" s="12" t="s">
+      <c r="M6" s="9" t="s">
         <v>38</v>
       </c>
       <c r="N6" s="3">
@@ -1228,7 +1217,7 @@
       </c>
       <c r="Q6" s="3"/>
     </row>
-    <row r="7" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>15</v>
       </c>
@@ -1294,19 +1283,19 @@
         <f t="shared" si="0"/>
         <v>Strong Order</v>
       </c>
-      <c r="M8" s="7" t="s">
+      <c r="M8" s="14" t="s">
         <v>39</v>
       </c>
-      <c r="N8" s="8"/>
+      <c r="N8" s="15"/>
       <c r="P8" s="5" t="s">
         <v>54</v>
       </c>
-      <c r="Q8" s="16">
+      <c r="Q8" s="11">
         <f>AVERAGEIF(Category,"Furniture",Profit)</f>
         <v>5857.1428571428569</v>
       </c>
     </row>
-    <row r="9" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
         <v>19</v>
       </c>
@@ -1335,7 +1324,7 @@
         <f t="shared" si="0"/>
         <v>Normal Order</v>
       </c>
-      <c r="M9" s="10" t="s">
+      <c r="M9" s="7" t="s">
         <v>40</v>
       </c>
       <c r="N9" s="3">
@@ -1345,12 +1334,12 @@
       <c r="P9" s="5" t="s">
         <v>55</v>
       </c>
-      <c r="Q9" s="15">
+      <c r="Q9" s="11">
         <f>AVERAGEIF(Category,"Electronics",Profit)</f>
         <v>9187.5</v>
       </c>
     </row>
-    <row r="10" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
         <v>20</v>
       </c>
@@ -1379,7 +1368,7 @@
         <f t="shared" si="0"/>
         <v>Normal Order</v>
       </c>
-      <c r="M10" s="10" t="s">
+      <c r="M10" s="7" t="s">
         <v>41</v>
       </c>
       <c r="N10" s="3">
@@ -1424,7 +1413,7 @@
         <v>Strong Order</v>
       </c>
     </row>
-    <row r="12" spans="1:17" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:17" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>22</v>
       </c>
@@ -1453,16 +1442,16 @@
         <f t="shared" si="0"/>
         <v>Normal Order</v>
       </c>
-      <c r="M12" s="10" t="s">
+      <c r="M12" s="7" t="s">
         <v>42</v>
       </c>
       <c r="N12" s="3"/>
-      <c r="P12" s="17" t="s">
+      <c r="P12" s="16" t="s">
         <v>56</v>
       </c>
-      <c r="Q12" s="17"/>
-    </row>
-    <row r="13" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+      <c r="Q12" s="16"/>
+    </row>
+    <row r="13" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>23</v>
       </c>
@@ -1491,7 +1480,7 @@
         <f t="shared" si="0"/>
         <v>Normal Order</v>
       </c>
-      <c r="M13" s="12" t="s">
+      <c r="M13" s="9" t="s">
         <v>45</v>
       </c>
       <c r="N13" s="3">
@@ -1506,7 +1495,7 @@
         <v>161000</v>
       </c>
     </row>
-    <row r="14" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>24</v>
       </c>
@@ -1535,7 +1524,7 @@
         <f t="shared" si="0"/>
         <v>Normal Order</v>
       </c>
-      <c r="M14" s="12" t="s">
+      <c r="M14" s="9" t="s">
         <v>46</v>
       </c>
       <c r="N14" s="3">
@@ -1550,7 +1539,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="15" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>25</v>
       </c>
@@ -1579,7 +1568,7 @@
         <f t="shared" si="0"/>
         <v>Normal Order</v>
       </c>
-      <c r="M15" s="12" t="s">
+      <c r="M15" s="9" t="s">
         <v>43</v>
       </c>
       <c r="N15" s="3">
@@ -1623,7 +1612,7 @@
         <f t="shared" si="0"/>
         <v>Strong Order</v>
       </c>
-      <c r="M16" s="12" t="s">
+      <c r="M16" s="9" t="s">
         <v>44</v>
       </c>
       <c r="N16" s="3">
@@ -1631,7 +1620,7 @@
         <v>128000</v>
       </c>
     </row>
-    <row r="17" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
         <v>27</v>
       </c>
@@ -1660,7 +1649,7 @@
         <f t="shared" si="0"/>
         <v>Normal Order</v>
       </c>
-      <c r="M17" s="12" t="s">
+      <c r="M17" s="9" t="s">
         <v>47</v>
       </c>
       <c r="N17" s="3">
@@ -1698,7 +1687,7 @@
         <v>Strong Order</v>
       </c>
     </row>
-    <row r="19" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
         <v>29</v>
       </c>
@@ -1728,7 +1717,7 @@
         <v>Normal Order</v>
       </c>
     </row>
-    <row r="20" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
         <v>30</v>
       </c>
@@ -1788,7 +1777,7 @@
         <v>Strong Order</v>
       </c>
     </row>
-    <row r="22" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
         <v>32</v>
       </c>
@@ -1819,18 +1808,6 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="H2:J22" xr:uid="{00000000-0001-0000-0000-000000000000}">
-    <filterColumn colId="0">
-      <filters>
-        <filter val="High Value"/>
-      </filters>
-    </filterColumn>
-    <filterColumn colId="1">
-      <filters>
-        <filter val="High Profit"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
   <mergeCells count="6">
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="M2:N2"/>

</xml_diff>